<commit_message>
Add T00 seed0 and ablations T01/T03/T05, update results and report
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/submissions/2A202602870_NguyenVanXuanLoc/results.xlsx
+++ b/submissions/2A202602870_NguyenVanXuanLoc/results.xlsx
@@ -827,7 +827,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U3"/>
+  <dimension ref="A1:U7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -944,7 +944,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -972,19 +972,19 @@
         <v>2</v>
       </c>
       <c r="J2" t="n">
-        <v>0.4738360943686613</v>
+        <v>0.4555424892456536</v>
       </c>
       <c r="K2" t="n">
-        <v>0.6680948300485575</v>
+        <v>0.6555269922879178</v>
       </c>
       <c r="L2" t="n">
-        <v>0.06475804360360636</v>
+        <v>0.07045908291696554</v>
       </c>
       <c r="M2" t="n">
-        <v>47.20521739299994</v>
+        <v>47.72177912399999</v>
       </c>
       <c r="N2" t="n">
-        <v>6.276749000051041</v>
+        <v>5.75279099999193</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -1017,7 +1017,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -1045,19 +1045,19 @@
         <v>2</v>
       </c>
       <c r="J3" t="n">
-        <v>0.4616580004057853</v>
+        <v>0.4738360943686613</v>
       </c>
       <c r="K3" t="n">
-        <v>0.6606683804627249</v>
+        <v>0.6680948300485575</v>
       </c>
       <c r="L3" t="n">
-        <v>0.06766010471241315</v>
+        <v>0.06475804360360636</v>
       </c>
       <c r="M3" t="n">
-        <v>48.46155525750004</v>
+        <v>47.20521739299994</v>
       </c>
       <c r="N3" t="n">
-        <v>6.349715500050479</v>
+        <v>6.276749000051041</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -1082,6 +1082,302 @@
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr"/>
       <c r="U3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>T00</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>resnet50</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>timm/resnet50.a1_in1k</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>23.53</v>
+      </c>
+      <c r="F4" t="n">
+        <v>4.09</v>
+      </c>
+      <c r="G4" t="n">
+        <v>224</v>
+      </c>
+      <c r="H4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I4" t="n">
+        <v>2</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.4616580004057853</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0.6606683804627249</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0.06766010471241315</v>
+      </c>
+      <c r="M4" t="n">
+        <v>48.46155525750004</v>
+      </c>
+      <c r="N4" t="n">
+        <v>6.349715500050479</v>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Tesla T4</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>2.11.0+cu128</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>basic</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>ce</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr"/>
+      <c r="T4" t="inlineStr"/>
+      <c r="U4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>T01</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>resnet50</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>timm/resnet50.a1_in1k</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>23.53</v>
+      </c>
+      <c r="F5" t="n">
+        <v>4.09</v>
+      </c>
+      <c r="G5" t="n">
+        <v>224</v>
+      </c>
+      <c r="H5" t="n">
+        <v>2</v>
+      </c>
+      <c r="I5" t="n">
+        <v>2</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0.4781849566169362</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0.09576303979596819</v>
+      </c>
+      <c r="M5" t="n">
+        <v>52.43539657400004</v>
+      </c>
+      <c r="N5" t="n">
+        <v>6.387668999991547</v>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Tesla T4</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>2.11.0+cu128</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>color</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>ce</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr"/>
+      <c r="T5" t="inlineStr"/>
+      <c r="U5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>T03</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>resnet50</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>timm/resnet50.a1_in1k</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>23.53</v>
+      </c>
+      <c r="F6" t="n">
+        <v>4.09</v>
+      </c>
+      <c r="G6" t="n">
+        <v>224</v>
+      </c>
+      <c r="H6" t="n">
+        <v>2</v>
+      </c>
+      <c r="I6" t="n">
+        <v>2</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0.4877689973270336</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0.6718080548414739</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0.1326235212895174</v>
+      </c>
+      <c r="M6" t="n">
+        <v>48.77127393099997</v>
+      </c>
+      <c r="N6" t="n">
+        <v>6.07130150001467</v>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Tesla T4</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>2.11.0+cu128</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>basic</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>ls</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr"/>
+      <c r="T6" t="inlineStr"/>
+      <c r="U6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>T05</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>resnet50</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>timm/resnet50.a1_in1k</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>23.53</v>
+      </c>
+      <c r="F7" t="n">
+        <v>4.09</v>
+      </c>
+      <c r="G7" t="n">
+        <v>224</v>
+      </c>
+      <c r="H7" t="n">
+        <v>2</v>
+      </c>
+      <c r="I7" t="n">
+        <v>2</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0.5476022186606897</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0.55641245358469</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0.04952607767858087</v>
+      </c>
+      <c r="M7" t="n">
+        <v>49.72433776</v>
+      </c>
+      <c r="N7" t="n">
+        <v>6.197876000015867</v>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>Tesla T4</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>2.11.0+cu128</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>basic</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>ce</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>balanced</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr"/>
+      <c r="U7" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1184,42 +1480,42 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>[1, 2]</t>
+          <t>[0, 1, 2]</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0.6679498146564016</v>
+        <v>0.6651458986788329</v>
       </c>
       <c r="E2" t="n">
-        <v>0.006250444886450779</v>
+        <v>0.006566571789531771</v>
       </c>
       <c r="F2" t="n">
-        <v>0.4699387807060643</v>
+        <v>0.4670367909106657</v>
       </c>
       <c r="G2" t="n">
-        <v>0.01174784644304297</v>
+        <v>0.009709303906174332</v>
       </c>
       <c r="H2" t="n">
-        <v>0.432764944977704</v>
+        <v>0.4300042491053566</v>
       </c>
       <c r="I2" t="n">
-        <v>0.01933546173720829</v>
+        <v>0.01448427994048409</v>
       </c>
       <c r="J2" t="n">
-        <v>0.06494653142571999</v>
+        <v>0.0674832867978329</v>
       </c>
       <c r="K2" t="n">
-        <v>0.01331186587862234</v>
+        <v>0.01038789054808752</v>
       </c>
       <c r="L2" t="n">
-        <v>0.9641524234180016</v>
+        <v>0.9754896010261209</v>
       </c>
       <c r="M2" t="n">
-        <v>0.00236092116833209</v>
+        <v>0.01970740375431695</v>
       </c>
     </row>
     <row r="3">
@@ -1385,13 +1681,13 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.1393805309734513</v>
+        <v>0.1312684365781711</v>
       </c>
       <c r="D2" t="n">
-        <v>0.03441670173916825</v>
+        <v>0.0281011192968402</v>
       </c>
       <c r="E2" t="n">
-        <v>0.2368046055631555</v>
+        <v>0.2250531995744034</v>
       </c>
       <c r="F2" t="n">
         <v>226</v>
@@ -1409,13 +1705,13 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.2957746478873239</v>
+        <v>0.3082942097026604</v>
       </c>
       <c r="D3" t="n">
-        <v>0.02655800117132572</v>
+        <v>0.02868591984322904</v>
       </c>
       <c r="E3" t="n">
-        <v>0.4245291612579991</v>
+        <v>0.4357076128816768</v>
       </c>
       <c r="F3" t="n">
         <v>213</v>
@@ -1433,13 +1729,13 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.748792270531401</v>
+        <v>0.7487922705314011</v>
       </c>
       <c r="D4" t="n">
-        <v>0.05465559661345296</v>
+        <v>0.03864734299516909</v>
       </c>
       <c r="E4" t="n">
-        <v>0.7309087868907282</v>
+        <v>0.7321382433931869</v>
       </c>
       <c r="F4" t="n">
         <v>207</v>
@@ -1457,13 +1753,13 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.01707317073170732</v>
+        <v>0.03252032520325204</v>
       </c>
       <c r="D5" t="n">
-        <v>0.003449301371641695</v>
+        <v>0.02686619779163952</v>
       </c>
       <c r="E5" t="n">
-        <v>0.03338042289464091</v>
+        <v>0.06111759134680097</v>
       </c>
       <c r="F5" t="n">
         <v>205</v>
@@ -1481,13 +1777,13 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.687793427230047</v>
+        <v>0.7089201877934271</v>
       </c>
       <c r="D6" t="n">
-        <v>0.08299375366039292</v>
+        <v>0.06915924818148468</v>
       </c>
       <c r="E6" t="n">
-        <v>0.6162320854995567</v>
+        <v>0.6147729518371806</v>
       </c>
       <c r="F6" t="n">
         <v>213</v>
@@ -1505,13 +1801,13 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.3267326732673267</v>
+        <v>0.3201320132013201</v>
       </c>
       <c r="D7" t="n">
-        <v>0.007001057239470774</v>
+        <v>0.01245847266546329</v>
       </c>
       <c r="E7" t="n">
-        <v>0.4706398230763364</v>
+        <v>0.4657206663646163</v>
       </c>
       <c r="F7" t="n">
         <v>202</v>
@@ -1529,13 +1825,13 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.4744186046511628</v>
+        <v>0.4310077519379845</v>
       </c>
       <c r="D8" t="n">
-        <v>0.006577737499409764</v>
+        <v>0.07533352318298504</v>
       </c>
       <c r="E8" t="n">
-        <v>0.559659475815557</v>
+        <v>0.5282425855541869</v>
       </c>
       <c r="F8" t="n">
         <v>215</v>
@@ -1553,13 +1849,13 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.2598039215686275</v>
+        <v>0.2467320261437909</v>
       </c>
       <c r="D9" t="n">
-        <v>0.0207972582701926</v>
+        <v>0.02699789483963777</v>
       </c>
       <c r="E9" t="n">
-        <v>0.3777930298177381</v>
+        <v>0.3633861834472653</v>
       </c>
       <c r="F9" t="n">
         <v>204</v>
@@ -1577,13 +1873,13 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0.9451152579582875</v>
+        <v>0.9423710208562021</v>
       </c>
       <c r="D10" t="n">
-        <v>0.009314249587528597</v>
+        <v>0.008122200102606322</v>
       </c>
       <c r="E10" t="n">
-        <v>0.7795016355388672</v>
+        <v>0.777192083796674</v>
       </c>
       <c r="F10" t="n">
         <v>1822</v>
@@ -2071,7 +2367,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.4699387807060643</v>
+        <v>0.4670367909106657</v>
       </c>
     </row>
   </sheetData>

</xml_diff>